<commit_message>
docs: add R-17 transport contract to the plan, policy and tasks (FE-17)
</commit_message>
<xml_diff>
--- a/doc/SWP391_Frontend_Tasks_R09_R16.xlsx
+++ b/doc/SWP391_Frontend_Tasks_R09_R16.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$K$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$K$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -874,36 +874,55 @@
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>R-17 Hợp đồng</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>COUNTIF(Tasks!$B$2:$B$500,A28)</f>
+        <v/>
+      </c>
+      <c r="C28">
+        <f>COUNTIFS(Tasks!$B$2:$B$500,A28,Tasks!$I$2:$I$500,"Xong")</f>
+        <v/>
+      </c>
+      <c r="D28" s="3">
+        <f>IF(B28=0,0,C28/B28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>• Nguồn: doc/TASKS_R09_R16.md (26/10/2026). Mô tả đầy đủ, tiêu chí hoàn thành và thứ tự làm nằm trong file .md.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>• Nghiệp vụ: PLAN_NGHIEP_VU_R09.md; chính sách gửi khách: CHINH_SACH_DICH_VU.md (cùng thư mục với file .md task).</t>
+          <t>• Nguồn: doc/TASKS_R09_R16.md (26/10/2026). Mô tả đầy đủ, tiêu chí hoàn thành và thứ tự làm nằm trong file .md.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>• Điểm = độ lớn tương đối: Cao 5, Trung bình 3, Thấp 2. Không phải số ngày.</t>
+          <t>• Nghiệp vụ: PLAN_NGHIEP_VU_R09.md; chính sách gửi khách: CHINH_SACH_DICH_VU.md (cùng thư mục với file .md task).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t>• Điểm = độ lớn tương đối: Cao 5, Trung bình 3, Thấp 2. Không phải số ngày.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>• Trạng thái hợp lệ: Chưa làm, Đang làm, Review, Xong.</t>
         </is>
@@ -920,7 +939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1809,9 +1828,60 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>FE-17</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>R-17 Hợp đồng</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Hợp đồng vận chuyển: xem trước, chấp nhận, tải PDF, chấp nhận bản mới</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Nút Xem hợp đồng (PDF); Chấp nhận &amp; đặt cọc chỉ bật khi đã mở hợp đồng và tích đã đọc, gửi contractId + mã băm. Khối Hợp đồng trên trang đơn (phiên bản, tải PDF, lịch sử). Thẻ Hợp đồng cần xác nhận lại khi có bản mới. Nhân sự xem / tải. Ô Air Waybill cho chuyến hàng không.</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Thiên</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>FE-05, BE-20</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Chi tiết: doc/TASKS_R09_R16.md mục FE-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K17"/>
-  <conditionalFormatting sqref="I2:I67">
+  <autoFilter ref="A1:K18"/>
+  <conditionalFormatting sqref="I2:I68">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Xong"</formula>
     </cfRule>
@@ -1823,10 +1893,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I2:I68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Chưa làm,Đang làm,Review,Xong"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Thiên,Vũ,Thắng"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>